<commit_message>
update TestCase doc and Defect doc
</commit_message>
<xml_diff>
--- a/20130199_TestCase.xlsx
+++ b/20130199_TestCase.xlsx
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="201">
   <si>
     <t>Module Code</t>
   </si>
@@ -154,7 +154,7 @@
     <t>Kiểm tra hiển thị các giá trị mặc định của các tiêu chí lọc ở giao diện rút gọn thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]</t>
   </si>
@@ -168,7 +168,7 @@
     <t>Kiểm tra hiển thị các tiêu chí lọc ở giao diện đầy đủ khi bấm vào nút [Tất cả] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước:
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.</t>
@@ -219,7 +219,7 @@
     <t>Kiểm tra chọn một giá trị trong một tiêu chí lọc thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -232,7 +232,7 @@
     <t>Kiểm tra chọn nhiều giá trị trong một tiêu chí lọc thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -245,7 +245,7 @@
     <t>Kiểm tra chọn một giá trị của mỗi tiêu chí lọc trong tất cả các tiêu chí lọc thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -255,7 +255,7 @@
     <t>Kiểm tra chọn nhiều giá trị của mỗi tiêu chí lọc trong tất cả tiêu chí lọc thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -279,13 +279,19 @@
     <t>Kiểm tra hiển thị các khoảng giá được đề xuất thành công.</t>
   </si>
   <si>
+    <t>Bước
+1. Truy cập website tiki.vn.
+2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
+3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.</t>
+  </si>
+  <si>
     <t>Trong tiêu chí giá, các mức giá đề xuất sẽ được hiển thị để người dùng lựa chọn.</t>
   </si>
   <si>
     <t>Kiểm tra khoảng giá hiển thị khi người dùng chọn vào khoảng giá được đề xuất thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -301,7 +307,7 @@
     <t>Kiểm tra nhập giá vào khoảng giá tùy chỉnh thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -314,7 +320,7 @@
     <t>Kiểm tra không cho phép nhập chữ vào ô nhập bên trái trong khoảng giá thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -328,7 +334,7 @@
     <t>Kiểm tra không cho phép nhập chữ vào ô nhập bên phải trong khoảng giá thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -341,7 +347,7 @@
     <t>Kiểm tra không cho phép nhập ký tự đặc biệt vào ô nhập bên trái trong khoảng giá thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -354,7 +360,7 @@
     <t>Kiểm tra không cho phép nhập ký tự đặc biệt vào ô nhập bên phải trong khoảng giá thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -367,7 +373,7 @@
     <t>Kiểm tra không cho phép giá trị nhập vào của ô bên trái lớn hơn ô bên phải trong khoảng giá thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -380,7 +386,7 @@
     <t>Kiểm tra không cho phép nhập giá trị của ô bên trái bằng với giá trị của ô bên phải trong khoảng giá thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -393,7 +399,7 @@
     <t>Kiểm tra xóa giá trị của khoảng giá khi bấm vào nút [Xóa] không thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc phía trên danh sách sản phẩm.
@@ -421,7 +427,7 @@
     <t>Lọc các sản phẩm có dịch vụ [Trả góp 0%] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -435,7 +441,7 @@
     <t>Lọc sản phẩm có dịch vụ [NOW Giao siêu tốc 2h] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -449,7 +455,7 @@
     <t>Lọc sản phẩm có dịch vụ [NOW Giao siêu tốc 2h] và [Trả góp 0%] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -463,7 +469,7 @@
     <t>Lọc sản phẩm được khuyến mãi [TOP DEAL Siêu rẻ] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -477,7 +483,7 @@
     <t>Lọc sản phẩm có khuyến mãi [FREESHIP XTRA] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -491,7 +497,7 @@
     <t>Lọc sản phẩm có khuyến mãi [FREESHIP XTRA] và [TOP DEAL Siêu rẻ] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -505,7 +511,7 @@
     <t>Lọc sản phẩm có đánh giá [từ 3 sao] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -516,10 +522,10 @@
     <t>Hiển thị các sản phẩm có đánh giá từ 3 sao trở lên.</t>
   </si>
   <si>
-    <t>Lọc sản phẩm có đánh giá [từ 4 sao] thất bại.</t>
+    <t>Lọc sản phẩm có đánh giá [từ 4 sao] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -527,10 +533,13 @@
 5. Nhấp vào nút [Xem kết quả].</t>
   </si>
   <si>
+    <t>Hiển thị các sản phẩm có đánh giá từ 4 sao trở lên.</t>
+  </si>
+  <si>
     <t>Lọc sản phẩm có đánh giá [từ 5 sao] thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -538,13 +547,13 @@
 5. Nhấp vào nút [Xem kết quả].</t>
   </si>
   <si>
-    <t>Hiển thị các sản phẩm có đánh giá từ 5 sao trở lên.</t>
+    <t>Hiển thị các sản phẩm có đánh giá 5 sao</t>
   </si>
   <si>
     <t>Lọc sản phẩm có giá dưới 2.000.000 thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -558,7 +567,7 @@
     <t>Lọc sản phẩm có giá từ 2.000.000 đến 4.000.000 thất bại.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -572,7 +581,7 @@
     <t>Lọc sản phẩm có giá từ 4.000.000 đến 12.000.000 thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -586,7 +595,7 @@
     <t>Lọc các sản phẩm có giá trên 12.000.000 thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -600,7 +609,7 @@
     <t>Lọc sản phẩm có giá dưới 200đ thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -614,7 +623,7 @@
     <t>Lọc sản phẩm có giá trên 100.200.000.000 thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -628,7 +637,7 @@
     <t>Lọc các sản phẩm có giá từ 1.200.000 đến 1.200.000 thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -642,7 +651,7 @@
     <t>Lọc các sản phẩm có giá từ 1.200.000 đến 2.200.000 thành công.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -656,7 +665,7 @@
     <t>Lọc các sản phẩm có giá từ 3.200.000 đến 1.200.000 thất bại.</t>
   </si>
   <si>
-    <t>Bước chân:
+    <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
@@ -2241,13 +2250,13 @@
     </dxf>
   </dxfs>
   <tableStyles count="2">
-    <tableStyle name="Login-Logout-style" pivot="0" count="4" xr9:uid="{4D36C29B-6CCC-4D7D-8DC9-F947B1C6689E}">
+    <tableStyle name="Login-Logout-style" pivot="0" count="4" xr9:uid="{ADBE22D0-4EA8-4ADE-8739-AFBD0DFF8961}">
       <tableStyleElement type="headerRow" dxfId="11"/>
       <tableStyleElement type="totalRow" dxfId="10"/>
       <tableStyleElement type="firstRowStripe" dxfId="9"/>
       <tableStyleElement type="secondRowStripe" dxfId="8"/>
     </tableStyle>
-    <tableStyle name="List Organisation-style" pivot="0" count="4" xr9:uid="{E1E23B39-ADFA-41D3-B1D6-5095A17DA949}">
+    <tableStyle name="List Organisation-style" pivot="0" count="4" xr9:uid="{97F2BE3B-BE3F-4B8B-800D-7B02A05412C6}">
       <tableStyleElement type="headerRow" dxfId="15"/>
       <tableStyleElement type="totalRow" dxfId="14"/>
       <tableStyleElement type="firstRowStripe" dxfId="13"/>
@@ -2674,15 +2683,15 @@
     <row r="6" customHeight="1" spans="1:26">
       <c r="A6" s="15">
         <f>COUNTIF(F9:F1210,"Passed")</f>
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B6" s="16">
         <f>COUNTIF(F9:F1210,"Failed")</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C6" s="16">
         <f>F6-E6-D6-B6-A6</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D6" s="16">
         <f>COUNTIF(F$9:F$1210,"Blocked")</f>
@@ -3271,10 +3280,10 @@
         <v>53</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="D20" s="26" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E20" s="31" t="s">
         <v>32</v>
@@ -3311,16 +3320,16 @@
         <v>[PDT_FLTR_Check_13]</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E21" s="31" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F21" s="27" t="s">
         <v>2</v>
@@ -3354,13 +3363,13 @@
         <v>[PDT_FLTR_Check_14]</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D22" s="26" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E22" s="31" t="s">
         <v>32</v>
@@ -3397,13 +3406,13 @@
         <v>[PDT_FLTR_Check_15]</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E23" s="31" t="s">
         <v>32</v>
@@ -3440,13 +3449,13 @@
         <v>[PDT_FLTR_Check_16]</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E24" s="31" t="s">
         <v>32</v>
@@ -3483,13 +3492,13 @@
         <v>[PDT_FLTR_Check_17]</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E25" s="31" t="s">
         <v>32</v>
@@ -3526,13 +3535,13 @@
         <v>[PDT_FLTR_Check_18]</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E26" s="31" t="s">
         <v>32</v>
@@ -3569,13 +3578,13 @@
         <v>[PDT_FLTR_Check_19]</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D27" s="26" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E27" s="31" t="s">
         <v>32</v>
@@ -3612,13 +3621,13 @@
         <v>[PDT_FLTR_Check_20]</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D28" s="26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E28" s="31" t="s">
         <v>32</v>
@@ -3655,13 +3664,13 @@
         <v>[PDT_FLTR_Check_21]</v>
       </c>
       <c r="B29" s="29" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D29" s="26" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E29" s="31" t="s">
         <v>32</v>
@@ -3698,13 +3707,13 @@
         <v>[PDT_FLTR_Check_22]</v>
       </c>
       <c r="B30" s="26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D30" s="26" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E30" s="31" t="s">
         <v>32</v>
@@ -3741,13 +3750,13 @@
         <v>[PDT_FLTR_Filter_23]</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E31" s="31" t="s">
         <v>32</v>
@@ -3784,13 +3793,13 @@
         <v>[PDT_FLTR_Filter_24]</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D32" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E32" s="31" t="s">
         <v>32</v>
@@ -3827,13 +3836,13 @@
         <v>[PDT_FLTR_Filter_25]</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D33" s="26" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E33" s="31" t="s">
         <v>32</v>
@@ -3870,13 +3879,13 @@
         <v>[PDT_FLTR_Filter_26]</v>
       </c>
       <c r="B34" s="26" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C34" s="26" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D34" s="26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E34" s="31" t="s">
         <v>32</v>
@@ -3913,13 +3922,13 @@
         <v>[PDT_FLTR_Filter_27]</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D35" s="26" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E35" s="31" t="s">
         <v>32</v>
@@ -3956,13 +3965,13 @@
         <v>[PDT_FLTR_Filter_28]</v>
       </c>
       <c r="B36" s="26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D36" s="26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E36" s="31" t="s">
         <v>32</v>
@@ -3999,13 +4008,13 @@
         <v>[PDT_FLTR_Filter_29]</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E37" s="31" t="s">
         <v>32</v>
@@ -4042,19 +4051,19 @@
         <v>[PDT_FLTR_Filter_30]</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C38" s="26" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D38" s="26" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E38" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F38" s="27" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G38" s="28">
         <v>45673</v>
@@ -4085,19 +4094,19 @@
         <v>[PDT_FLTR_Filter_31]</v>
       </c>
       <c r="B39" s="26" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D39" s="26" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E39" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G39" s="28">
         <v>45673</v>
@@ -4128,19 +4137,19 @@
         <v>[PDT_FLTR_Filter_32]</v>
       </c>
       <c r="B40" s="26" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D40" s="26" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E40" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G40" s="28">
         <v>45673</v>
@@ -4171,13 +4180,13 @@
         <v>[PDT_FLTR_Filter_33]</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D41" s="26" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E41" s="31" t="s">
         <v>32</v>
@@ -4214,19 +4223,19 @@
         <v>[PDT_FLTR_Filter_34]</v>
       </c>
       <c r="B42" s="26" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D42" s="26" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E42" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F42" s="27" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G42" s="28">
         <v>45673</v>
@@ -4257,19 +4266,19 @@
         <v>[PDT_FLTR_Filter_35]</v>
       </c>
       <c r="B43" s="26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D43" s="26" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E43" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F43" s="27" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G43" s="28">
         <v>45673</v>
@@ -4300,13 +4309,13 @@
         <v>[PDT_FLTR_Filter_36]</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C44" s="26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D44" s="26" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E44" s="31" t="s">
         <v>32</v>
@@ -4343,13 +4352,13 @@
         <v>[PDT_FLTR_Filter_37]</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C45" s="26" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D45" s="26" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E45" s="31" t="s">
         <v>32</v>
@@ -4386,19 +4395,19 @@
         <v>[PDT_FLTR_Filter_38]</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C46" s="26" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D46" s="26" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E46" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G46" s="28">
         <v>45673</v>
@@ -4429,13 +4438,13 @@
         <v>[PDT_FLTR_Filter_39]</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D47" s="26" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E47" s="31" t="s">
         <v>32</v>
@@ -4472,13 +4481,13 @@
         <v>[PDT_FLTR_Filter_40]</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C48" s="26" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D48" s="26" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E48" s="31" t="s">
         <v>32</v>
@@ -4515,13 +4524,13 @@
         <v>[PDT_FLTR_Filter_41]</v>
       </c>
       <c r="B49" s="26" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C49" s="26" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D49" s="26" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E49" s="31" t="s">
         <v>32</v>
@@ -4558,19 +4567,19 @@
         <v>[PDT_FLTR_Filter_42]</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C50" s="26" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D50" s="26" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E50" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F50" s="27" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G50" s="28">
         <v>45673</v>
@@ -4601,13 +4610,13 @@
         <v>[PDT_FLTR_Filter_43]</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C51" s="26" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D51" s="26" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E51" s="31" t="s">
         <v>32</v>
@@ -4644,13 +4653,13 @@
         <v>[PDT_FLTR_Filter_44]</v>
       </c>
       <c r="B52" s="26" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C52" s="26" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D52" s="26" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E52" s="31" t="s">
         <v>32</v>
@@ -4687,13 +4696,13 @@
         <v>[PDT_FLTR_Filter_45]</v>
       </c>
       <c r="B53" s="26" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C53" s="26" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D53" s="26" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E53" s="31" t="s">
         <v>32</v>
@@ -4730,13 +4739,13 @@
         <v>[PDT_FLTR_Filter_46]</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C54" s="26" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D54" s="26" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E54" s="31" t="s">
         <v>32</v>
@@ -4773,13 +4782,13 @@
         <v>[PDT_FLTR_Filter_47]</v>
       </c>
       <c r="B55" s="26" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C55" s="26" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D55" s="26" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E55" s="31" t="s">
         <v>32</v>
@@ -4816,19 +4825,19 @@
         <v>[PDT_FLTR_Filter_48]</v>
       </c>
       <c r="B56" s="26" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C56" s="26" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D56" s="26" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E56" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F56" s="27" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G56" s="28">
         <v>45673</v>
@@ -4859,19 +4868,19 @@
         <v>[PDT_FLTR_Filter_49]</v>
       </c>
       <c r="B57" s="26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C57" s="26" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D57" s="26" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E57" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F57" s="27" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G57" s="28">
         <v>45673</v>
@@ -4902,13 +4911,13 @@
         <v>[PDT_FLTR_Filter_50]</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C58" s="26" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D58" s="26" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E58" s="31" t="s">
         <v>32</v>
@@ -4945,13 +4954,13 @@
         <v>[PDT_FLTR_Filter_51]</v>
       </c>
       <c r="B59" s="26" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C59" s="26" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D59" s="26" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E59" s="31" t="s">
         <v>32</v>
@@ -4988,19 +4997,19 @@
         <v>[PDT_FLTR_Filter_52]</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C60" s="26" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D60" s="26" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E60" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F60" s="27" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G60" s="28">
         <v>45673</v>
@@ -5031,19 +5040,19 @@
         <v>[PDT_FLTR_Filter_53]</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C61" s="26" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D61" s="26" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E61" s="31" t="s">
         <v>32</v>
       </c>
       <c r="F61" s="27" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G61" s="28">
         <v>45673</v>
@@ -5074,13 +5083,13 @@
         <v>[PDT_FLTR_Filter_54]</v>
       </c>
       <c r="B62" s="26" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C62" s="26" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D62" s="26" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E62" s="31" t="s">
         <v>32</v>
@@ -5117,13 +5126,13 @@
         <v>[PDT_FLTR_Filter_55]</v>
       </c>
       <c r="B63" s="26" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C63" s="26" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D63" s="26" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E63" s="31" t="s">
         <v>32</v>
@@ -5160,13 +5169,13 @@
         <v>[PDT_FLTR_Filter_56]</v>
       </c>
       <c r="B64" s="26" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C64" s="26" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D64" s="26" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E64" s="31" t="s">
         <v>32</v>
@@ -5203,13 +5212,13 @@
         <v>[PDT_FLTR_Filter_57]</v>
       </c>
       <c r="B65" s="26" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C65" s="26" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D65" s="26" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E65" s="31" t="s">
         <v>32</v>
@@ -5246,13 +5255,13 @@
         <v>[PDT_FLTR_Filter_58]</v>
       </c>
       <c r="B66" s="26" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C66" s="26" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D66" s="26" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E66" s="31" t="s">
         <v>32</v>
@@ -5289,13 +5298,13 @@
         <v>[PDT_FLTR_Filter_59]</v>
       </c>
       <c r="B67" s="26" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C67" s="26" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D67" s="26" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E67" s="31" t="s">
         <v>32</v>
@@ -5332,13 +5341,13 @@
         <v>[PDT_FLTR_Filter_60]</v>
       </c>
       <c r="B68" s="26" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C68" s="26" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D68" s="26" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E68" s="31" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
update Q&A doc, testCase doc, testDesign doc
</commit_message>
<xml_diff>
--- a/20130199_TestCase.xlsx
+++ b/20130199_TestCase.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="27945" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="ProductsFilter" sheetId="5" r:id="rId1"/>
@@ -620,14 +620,14 @@
     <t>Hiển thị các sản phẩm có giá dưới 200 đ.</t>
   </si>
   <si>
-    <t>Lọc sản phẩm có giá trên 100.200.000.000 thành công.</t>
+    <t>Lọc sản phẩm có giá trên 9.200.000.000 thành công.</t>
   </si>
   <si>
     <t>Bước
 1. Truy cập website tiki.vn.
 2. Tại trang chủ chọn menu [Điện thoại - Máy tính bảng]
 3. Nhấp vào nút [Tất cả] trên menu bộ lọc ở phía trên danh sách sản phẩm.
-4. Trong phần tiêu chí [Giá], tiêu đề [Tự nhập khoảng giá], nhập 100200000000 vào ô bên trái, để trống ô bên phải.
+4. Trong phần tiêu chí [Giá], tiêu đề [Tự nhập khoảng giá], nhập 9200000000 vào ô bên trái, để trống ô bên phải.
 5. nhấp vào nút [Xem kết quả].</t>
   </si>
   <si>
@@ -2250,13 +2250,13 @@
     </dxf>
   </dxfs>
   <tableStyles count="2">
-    <tableStyle name="Login-Logout-style" pivot="0" count="4" xr9:uid="{ADBE22D0-4EA8-4ADE-8739-AFBD0DFF8961}">
+    <tableStyle name="Login-Logout-style" pivot="0" count="4" xr9:uid="{D34E80E0-7899-40FF-ACD6-D5C99312E823}">
       <tableStyleElement type="headerRow" dxfId="11"/>
       <tableStyleElement type="totalRow" dxfId="10"/>
       <tableStyleElement type="firstRowStripe" dxfId="9"/>
       <tableStyleElement type="secondRowStripe" dxfId="8"/>
     </tableStyle>
-    <tableStyle name="List Organisation-style" pivot="0" count="4" xr9:uid="{97F2BE3B-BE3F-4B8B-800D-7B02A05412C6}">
+    <tableStyle name="List Organisation-style" pivot="0" count="4" xr9:uid="{878C1ED8-DF9C-4078-85B4-7330D905624A}">
       <tableStyleElement type="headerRow" dxfId="15"/>
       <tableStyleElement type="totalRow" dxfId="14"/>
       <tableStyleElement type="firstRowStripe" dxfId="13"/>
@@ -2488,7 +2488,7 @@
   <dimension ref="A1:Z1214"/>
   <sheetFormatPr defaultColWidth="14.4285714285714" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.4285714285714" style="1" customWidth="1"/>
     <col min="2" max="2" width="23" style="1" customWidth="1"/>
     <col min="3" max="3" width="30.4285714285714" style="1" customWidth="1"/>
     <col min="4" max="4" width="32.5714285714286" style="1" customWidth="1"/>

</xml_diff>